<commit_message>
Add ownership checks to restrict proposal modification and deletion
Introduces `server/projectAccessControl.ts` with `userCanAccessProject` function. Modifies `server/projectRoutes.ts` to implement ownership checks on PATCH, DELETE, and POST bulk delete endpoints for proposal log entries, ensuring users can only modify/delete their own projects unless they are administrators.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 9c382587-0d27-441d-9d75-eab518567578
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/MU7Lv70
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-06.xlsx
+++ b/backups/proposal-log-2026-04-06.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="101">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -296,6 +296,24 @@
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69c42fb71e34da5627943f29</t>
+  </si>
+  <si>
+    <t>26-0215</t>
+  </si>
+  <si>
+    <t>33P Affordable Housing Multi-Family Devlopment</t>
+  </si>
+  <si>
+    <t>Residential</t>
+  </si>
+  <si>
+    <t>2026-04-15</t>
+  </si>
+  <si>
+    <t>Jon Smith</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69d046a028ff4e0032ca893c</t>
   </si>
 </sst>
 </file>
@@ -694,7 +712,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1282,8 +1300,52 @@
         <v>94</v>
       </c>
     </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>95</v>
+      </c>
+      <c r="B14" t="s">
+        <v>96</v>
+      </c>
+      <c r="C14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" t="s">
+        <v>97</v>
+      </c>
+      <c r="E14" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" t="s">
+        <v>98</v>
+      </c>
+      <c r="G14" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" t="s">
+        <v>99</v>
+      </c>
+      <c r="I14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J14" t="s">
+        <v>56</v>
+      </c>
+      <c r="K14" t="s">
+        <v>17</v>
+      </c>
+      <c r="L14" t="s">
+        <v>17</v>
+      </c>
+      <c r="M14" t="s">
+        <v>17</v>
+      </c>
+      <c r="N14" t="s">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N13"/>
+  <autoFilter ref="A1:N14"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update proposal log backup file with latest data
Update the proposal log backup file in the backups directory.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 64d3b0a0-3d56-4129-ac83-5afef245c13f
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/OqfnNVA
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-06.xlsx
+++ b/backups/proposal-log-2026-04-06.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="102">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -257,6 +257,9 @@
   </si>
   <si>
     <t>26-0208</t>
+  </si>
+  <si>
+    <t>GT</t>
   </si>
   <si>
     <t>26-0207</t>
@@ -1188,7 +1191,7 @@
         <v>19</v>
       </c>
       <c r="G11" t="s">
-        <v>17</v>
+        <v>82</v>
       </c>
       <c r="H11" t="s">
         <v>20</v>
@@ -1214,13 +1217,13 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D12" t="s">
         <v>76</v>
@@ -1229,13 +1232,13 @@
         <v>18</v>
       </c>
       <c r="F12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G12" t="s">
         <v>17</v>
       </c>
       <c r="H12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I12" t="s">
         <v>17</v>
@@ -1253,33 +1256,33 @@
         <v>17</v>
       </c>
       <c r="N12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C13" t="s">
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G13" t="s">
         <v>17</v>
       </c>
       <c r="H13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I13" t="s">
         <v>17</v>
@@ -1297,33 +1300,33 @@
         <v>17</v>
       </c>
       <c r="N13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C14" t="s">
         <v>26</v>
       </c>
       <c r="D14" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E14" t="s">
         <v>54</v>
       </c>
       <c r="F14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G14" t="s">
         <v>17</v>
       </c>
       <c r="H14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I14" t="s">
         <v>17</v>
@@ -1341,7 +1344,7 @@
         <v>17</v>
       </c>
       <c r="N14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>